<commit_message>
Finishing creating the graph and finalizing the data
</commit_message>
<xml_diff>
--- a/DCI_DCO_summary.xlsx
+++ b/DCI_DCO_summary.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -362,42 +362,82 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>room_count_mean</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>room_count_median</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>total_stays_mean</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>total_stays_median</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>dci_complete_mean</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>dci_complete_median</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>dci_complete_sd</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>dci_complete_var</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>dk_request_mean</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>dk_request_median</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dk_provisions_mean</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>dk_provisions_median</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>dk_succesful_stays_mean</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>dk_succesful_stays_median</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>dk_error_stays_mean</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>dk_error_stays_median</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>dco_completes_mean</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>dco_completes_median</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>dco_completes_sd</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>dco_completes_var</t>
         </is>
       </c>
     </row>
@@ -408,28 +448,52 @@
         </is>
       </c>
       <c r="B2">
+        <v>414.91</v>
+      </c>
+      <c r="C2">
+        <v>400</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>0.86</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>0.35</v>
-      </c>
-      <c r="E2">
-        <v>0.12</v>
-      </c>
-      <c r="F2">
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>0.92</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>0.88</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>0.51</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>0.04</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
         <v>0.21</v>
       </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0.4</v>
-      </c>
-      <c r="I2">
-        <v>0.16</v>
+      <c r="Q2">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -439,28 +503,52 @@
         </is>
       </c>
       <c r="B3">
+        <v>370.29</v>
+      </c>
+      <c r="C3">
+        <v>325</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>0.89</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>0.31</v>
-      </c>
-      <c r="E3">
-        <v>0.1</v>
-      </c>
-      <c r="F3">
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>0.93</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>0.89</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>0.48</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0.02</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
         <v>0.35</v>
       </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0.48</v>
-      </c>
-      <c r="I3">
-        <v>0.23</v>
+      <c r="Q3">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -470,28 +558,52 @@
         </is>
       </c>
       <c r="B4">
+        <v>1746.09</v>
+      </c>
+      <c r="C4">
+        <v>1610</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
         <v>0.74</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>0.44</v>
-      </c>
-      <c r="E4">
-        <v>0.19</v>
-      </c>
-      <c r="F4">
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>0.84</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>0.54</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+      <c r="N4">
+        <v>0.02</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
         <v>0.46</v>
       </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0.5</v>
-      </c>
-      <c r="I4">
-        <v>0.25</v>
+      <c r="Q4">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -501,28 +613,52 @@
         </is>
       </c>
       <c r="B5">
+        <v>634.64</v>
+      </c>
+      <c r="C5">
+        <v>656</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
         <v>0.75</v>
       </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>0.43</v>
-      </c>
-      <c r="E5">
-        <v>0.19</v>
-      </c>
-      <c r="F5">
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>0.84</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>0.79</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>0.46</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0.02</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
         <v>0.4</v>
       </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>0.49</v>
-      </c>
-      <c r="I5">
-        <v>0.24</v>
+      <c r="Q5">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -532,28 +668,52 @@
         </is>
       </c>
       <c r="B6">
+        <v>517.33</v>
+      </c>
+      <c r="C6">
+        <v>463</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
         <v>0.73</v>
       </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>0.45</v>
-      </c>
-      <c r="E6">
-        <v>0.2</v>
-      </c>
-      <c r="F6">
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>0.84</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>0.49</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0.02</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
         <v>0.33</v>
       </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0.47</v>
-      </c>
-      <c r="I6">
-        <v>0.22</v>
+      <c r="Q6">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>